<commit_message>
fix: configurando salvamento de dados no excel
</commit_message>
<xml_diff>
--- a/data/output/Reconciliation.xlsx
+++ b/data/output/Reconciliation.xlsx
@@ -1,13 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://suzano-my.sharepoint.com/personal/julianobs_suzano_com_br/Documents/Area Dev/GitHub/UiPath/LANCAMENTO_NFe/data/output/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_AD4D361C20488DEA4E38A073FC9B5C745BDEDD83" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54C6B3E1-B51A-41C8-8E98-B5AD3441D6DF}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Plan1" sheetId="1" r:id="rId1"/>
+    <sheet name="Invoices" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -19,7 +25,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -330,7 +336,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>

<commit_message>
fix: adiciona cabeçalhos ao excel e teste de preenchimento tabela
</commit_message>
<xml_diff>
--- a/data/output/Reconciliation.xlsx
+++ b/data/output/Reconciliation.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://suzano-my.sharepoint.com/personal/julianobs_suzano_com_br/Documents/Area Dev/GitHub/UiPath/LANCAMENTO_NFe/data/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_AD4D361C20488DEA4E38A073FC9B5C745BDEDD83" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54C6B3E1-B51A-41C8-8E98-B5AD3441D6DF}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_AD4D361C20488DEA4E38A073FC9B5C745BDEDD83" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F55F6E7F-0238-48D9-A9A8-5050DA596A0A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,6 +22,30 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Account Name
+</t>
+  </si>
+  <si>
+    <t>Contact Email</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -55,8 +79,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -72,6 +97,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -337,9 +366,38 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>